<commit_message>
[MOD] Actualizaciones en Taquilla y Dagas
- Taquilla:
  * Audio de explicación actualizado con los 15 clientes
  * Costo de entrada de niños cambiado a 4 + restricción de pago completo
  * Al responder incorrectamente ahora avanza al siguiente cliente

- Dagas:
  * Cambiado de 120s tiempo total/10s por ronda a 15 rondas totales
  * Al responder incorrectamente ahora avanza a la siguiente ronda
</commit_message>
<xml_diff>
--- a/assets/audios_tutor/audios_pepe/audios_pepe.xlsx
+++ b/assets/audios_tutor/audios_pepe/audios_pepe.xlsx
@@ -37,19 +37,19 @@
     <t>¡Hola! Soy Pepe. Bienvenido a la taquilla. Tu misión es vender entradas para el circo.</t>
   </si>
   <si>
-    <t>Las tarifas son: 3 Bs para los NIÑOS y 7 Bs para los ADULTOS. ¡Memorízalo bien!</t>
-  </si>
-  <si>
     <t>Calcula el total y mira cuánto paga el cliente. Si sobra dinero, debes dar VUELTO.</t>
   </si>
   <si>
     <t>Jala la PALANCA para abrir la caja y haz clic en las monedas para sumar el vuelto exacto.</t>
   </si>
   <si>
-    <t>Tienes 120 segundos. ¡Gana PUNTOS por cada venta correcta antes de que se acabe el TIEMPO!</t>
-  </si>
-  <si>
     <t>Cuando termines, jala la PALANCA de nuevo para confirmar. (Haz clic para empezar)</t>
+  </si>
+  <si>
+    <t>Debes atender a 15 clientes. ¡Gana PUNTOS por cada venta correcta!</t>
+  </si>
+  <si>
+    <t>Las tarifas son: 4 Bs para los NIÑOS y 7 Bs para los ADULTOS. ¡Memorízalo bien!</t>
   </si>
 </sst>
 </file>
@@ -419,7 +419,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -427,7 +427,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -435,7 +435,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -451,7 +451,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>